<commit_message>
Ratesheet update with two areas
</commit_message>
<xml_diff>
--- a/data/raw/The Vietnam DMC Data Mart.xlsx
+++ b/data/raw/The Vietnam DMC Data Mart.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="80">
   <si>
     <t>city</t>
   </si>
@@ -53,10 +53,10 @@
     <t>Hanoi</t>
   </si>
   <si>
-    <t>hotel_name_1</t>
-  </si>
-  <si>
-    <t>room_name_1</t>
+    <t>hanoi_hotel_1</t>
+  </si>
+  <si>
+    <t>hanoi_hotel_1_room_1</t>
   </si>
   <si>
     <t>CP</t>
@@ -65,7 +65,19 @@
     <t>MAP</t>
   </si>
   <si>
-    <t>room_name_2</t>
+    <t>hanoi_hotel_1_room_2</t>
+  </si>
+  <si>
+    <t>Da Nang</t>
+  </si>
+  <si>
+    <t>danang_hotel_1</t>
+  </si>
+  <si>
+    <t>danang_hotel_1_room_1</t>
+  </si>
+  <si>
+    <t>danang_hotel_1_room_2</t>
   </si>
   <si>
     <t>airport</t>
@@ -515,7 +527,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="5.38"/>
+    <col customWidth="1" min="1" max="1" width="10.0"/>
     <col customWidth="1" min="2" max="2" width="11.5"/>
     <col customWidth="1" min="3" max="3" width="11.75"/>
     <col customWidth="1" min="4" max="4" width="9.13"/>
@@ -690,6 +702,120 @@
         <v>46023.0</v>
       </c>
       <c r="L4" s="3">
+        <v>46387.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F5" s="2">
+        <v>10.0</v>
+      </c>
+      <c r="G5" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="H5" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I5" s="3">
+        <v>46023.0</v>
+      </c>
+      <c r="J5" s="3">
+        <v>46387.0</v>
+      </c>
+      <c r="K5" s="3">
+        <v>46023.0</v>
+      </c>
+      <c r="L5" s="3">
+        <v>46387.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F6" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>8.0</v>
+      </c>
+      <c r="H6" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="I6" s="3">
+        <v>46023.0</v>
+      </c>
+      <c r="J6" s="3">
+        <v>46387.0</v>
+      </c>
+      <c r="K6" s="3">
+        <v>46023.0</v>
+      </c>
+      <c r="L6" s="3">
+        <v>46387.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F7" s="2">
+        <v>8.0</v>
+      </c>
+      <c r="G7" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="I7" s="3">
+        <v>46023.0</v>
+      </c>
+      <c r="J7" s="3">
+        <v>46387.0</v>
+      </c>
+      <c r="K7" s="3">
+        <v>46023.0</v>
+      </c>
+      <c r="L7" s="3">
         <v>46387.0</v>
       </c>
     </row>
@@ -720,25 +846,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>8</v>
@@ -769,22 +895,22 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G2" s="2">
         <v>13.0</v>
@@ -804,22 +930,22 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G3" s="2">
         <v>84.0</v>
@@ -839,22 +965,22 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="F4" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G4" s="2">
         <v>74.0</v>
@@ -874,22 +1000,22 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G5" s="2">
         <v>14.0</v>
@@ -909,22 +1035,22 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G6" s="2">
         <v>84.0</v>
@@ -944,22 +1070,22 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E7" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G7" s="2">
         <v>74.0</v>
@@ -979,22 +1105,22 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E8" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G8" s="2">
         <v>7.0</v>
@@ -1014,22 +1140,22 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E9" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G9" s="2">
         <v>89.0</v>
@@ -1049,22 +1175,22 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E10" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G10" s="2">
         <v>76.0</v>
@@ -1084,22 +1210,22 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E11" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G11" s="2">
         <v>102.0</v>
@@ -1119,22 +1245,22 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E12" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G12" s="2">
         <v>10.0</v>
@@ -1154,22 +1280,22 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G13" s="2">
         <v>115.0</v>
@@ -1189,22 +1315,22 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E14" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G14" s="2">
         <v>119.0</v>
@@ -1224,22 +1350,22 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E15" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G15" s="2">
         <v>115.0</v>
@@ -1259,22 +1385,22 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E16" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G16" s="2">
         <v>119.0</v>
@@ -1294,22 +1420,22 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E17" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G17" s="2">
         <v>20.0</v>
@@ -1329,22 +1455,22 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G18" s="2">
         <v>3.0</v>
@@ -1364,22 +1490,22 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G19" s="2">
         <v>26.0</v>
@@ -1399,22 +1525,22 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G20" s="2">
         <v>0.0</v>
@@ -1434,22 +1560,22 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G21" s="2">
         <v>4.0</v>
@@ -1469,22 +1595,22 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G22" s="2">
         <v>4.0</v>
@@ -1504,22 +1630,22 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G23" s="2">
         <v>7.0</v>
@@ -1539,22 +1665,22 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G24" s="2">
         <v>7.0</v>
@@ -1574,22 +1700,22 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G25" s="2">
         <v>33.0</v>
@@ -1609,22 +1735,22 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G26" s="2">
         <v>41.0</v>
@@ -1644,22 +1770,22 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G27" s="2">
         <v>50.0</v>
@@ -1679,22 +1805,22 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G28" s="2">
         <v>12.0</v>
@@ -1714,22 +1840,22 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G29" s="2">
         <v>16.0</v>
@@ -1749,22 +1875,22 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G30" s="2">
         <v>13.0</v>
@@ -1784,22 +1910,22 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G31" s="2">
         <v>17.0</v>
@@ -1819,22 +1945,22 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G32" s="2">
         <v>28.0</v>
@@ -1854,22 +1980,22 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G33" s="2">
         <v>24.0</v>
@@ -1889,22 +2015,22 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G34" s="2">
         <v>32.0</v>
@@ -1924,22 +2050,22 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G35" s="2">
         <v>28.0</v>
@@ -1959,22 +2085,22 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G36" s="2">
         <v>41.0</v>
@@ -1994,22 +2120,22 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G37" s="2">
         <v>45.0</v>
@@ -2029,22 +2155,22 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G38" s="2">
         <v>48.0</v>
@@ -2064,22 +2190,22 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G39" s="2">
         <v>31.0</v>
@@ -2099,22 +2225,22 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G40" s="2">
         <v>35.0</v>
@@ -2134,22 +2260,22 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G41" s="2">
         <v>35.0</v>
@@ -2169,22 +2295,22 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G42" s="2">
         <v>39.0</v>
@@ -2204,22 +2330,22 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G43" s="2">
         <v>31.0</v>
@@ -2239,22 +2365,22 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G44" s="2">
         <v>35.0</v>

</xml_diff>